<commit_message>
feat: Import TMC rings, homepage bespoke journey, and launch pages
Ship 13 client-selected TMC rings into the catalog with Lab Prices, add the TMC review tooling, bespoke timeline strip, Privé/waitlist flows, and legal/FAQ pages for production.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/Inventory /Engagement Ring Prices/Lab Prices.xlsx
+++ b/public/Inventory /Engagement Ring Prices/Lab Prices.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="47">
   <si>
     <t>Name</t>
   </si>
@@ -70,6 +70,30 @@
     <t>Seraphina</t>
   </si>
   <si>
+    <t>Ophellia</t>
+  </si>
+  <si>
+    <t>Amarante</t>
+  </si>
+  <si>
+    <t>Anastasia</t>
+  </si>
+  <si>
+    <t>Noémi</t>
+  </si>
+  <si>
+    <t>Isolde</t>
+  </si>
+  <si>
+    <t>Nala</t>
+  </si>
+  <si>
+    <t>Elodie</t>
+  </si>
+  <si>
+    <t>Callista</t>
+  </si>
+  <si>
     <t>Vow &amp; Veil</t>
   </si>
   <si>
@@ -89,6 +113,21 @@
   </si>
   <si>
     <t>Radiant / Pear</t>
+  </si>
+  <si>
+    <t>Arabella</t>
+  </si>
+  <si>
+    <t>Evermore</t>
+  </si>
+  <si>
+    <t>Lumina</t>
+  </si>
+  <si>
+    <t>Vivienne</t>
+  </si>
+  <si>
+    <t>Sorella</t>
   </si>
   <si>
     <t>Ovalis</t>
@@ -745,7 +784,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>8</v>
@@ -754,7 +793,7 @@
         <v>15</v>
       </c>
       <c r="E22" s="3">
-        <v>2489.0</v>
+        <v>1799.0</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>10</v>
@@ -765,7 +804,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>11</v>
@@ -774,7 +813,7 @@
         <v>15</v>
       </c>
       <c r="E23" s="3">
-        <v>3389.0</v>
+        <v>2299.0</v>
       </c>
     </row>
     <row r="24">
@@ -782,7 +821,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>12</v>
@@ -791,7 +830,7 @@
         <v>15</v>
       </c>
       <c r="E24" s="3">
-        <v>4049.0</v>
+        <v>2799.0</v>
       </c>
     </row>
     <row r="25">
@@ -799,7 +838,7 @@
         <v>19</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>13</v>
@@ -808,15 +847,15 @@
         <v>15</v>
       </c>
       <c r="E25" s="3">
-        <v>4949.0</v>
+        <v>3299.0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>8</v>
@@ -825,18 +864,18 @@
         <v>15</v>
       </c>
       <c r="E27" s="3">
-        <v>2449.0</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>17</v>
+        <v>1875.0</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>11</v>
@@ -845,15 +884,15 @@
         <v>15</v>
       </c>
       <c r="E28" s="3">
-        <v>2949.0</v>
+        <v>2375.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>12</v>
@@ -862,15 +901,15 @@
         <v>15</v>
       </c>
       <c r="E29" s="3">
-        <v>3599.0</v>
+        <v>2875.0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>13</v>
@@ -879,27 +918,24 @@
         <v>15</v>
       </c>
       <c r="E30" s="3">
-        <v>4099.0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5"/>
+        <v>3375.0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E32" s="3">
-        <v>1949.0</v>
+        <v>2025.0</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>10</v>
@@ -907,61 +943,61 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E33" s="3">
-        <v>2449.0</v>
+        <v>2525.0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E34" s="3">
-        <v>3099.0</v>
+        <v>3025.0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E35" s="3">
-        <v>3599.0</v>
+        <v>3525.0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>8</v>
@@ -970,7 +1006,7 @@
         <v>15</v>
       </c>
       <c r="E37" s="3">
-        <v>2689.0</v>
+        <v>1899.0</v>
       </c>
       <c r="G37" s="4" t="s">
         <v>10</v>
@@ -978,10 +1014,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>11</v>
@@ -990,15 +1026,15 @@
         <v>15</v>
       </c>
       <c r="E38" s="3">
-        <v>3589.0</v>
+        <v>2399.0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>12</v>
@@ -1007,15 +1043,15 @@
         <v>15</v>
       </c>
       <c r="E39" s="3">
-        <v>4249.0</v>
+        <v>2899.0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>13</v>
@@ -1024,24 +1060,24 @@
         <v>15</v>
       </c>
       <c r="E40" s="3">
-        <v>5149.0</v>
+        <v>3399.0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E42" s="3">
-        <v>2179.0</v>
+        <v>2149.0</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>10</v>
@@ -1049,61 +1085,61 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E43" s="3">
-        <v>2679.0</v>
+        <v>2649.0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E44" s="3">
-        <v>3329.0</v>
+        <v>3299.0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E45" s="3">
-        <v>3729.0</v>
+        <v>3799.0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>8</v>
@@ -1112,18 +1148,18 @@
         <v>15</v>
       </c>
       <c r="E47" s="3">
-        <v>2379.0</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>17</v>
+        <v>1600.0</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>11</v>
@@ -1132,15 +1168,15 @@
         <v>15</v>
       </c>
       <c r="E48" s="3">
-        <v>2879.0</v>
+        <v>2100.0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>12</v>
@@ -1149,15 +1185,15 @@
         <v>15</v>
       </c>
       <c r="E49" s="3">
-        <v>3529.0</v>
+        <v>2600.0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>13</v>
@@ -1166,86 +1202,86 @@
         <v>15</v>
       </c>
       <c r="E50" s="3">
-        <v>3929.0</v>
+        <v>3100.0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E52" s="3">
-        <v>2635.0</v>
-      </c>
-      <c r="G52" s="6" t="s">
-        <v>17</v>
+        <v>2495.0</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E53" s="3">
-        <v>3135.0</v>
+        <v>2995.0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E54" s="3">
-        <v>3635.0</v>
+        <v>3495.0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E55" s="3">
-        <v>4135.0</v>
+        <v>3995.0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>8</v>
@@ -1254,18 +1290,18 @@
         <v>15</v>
       </c>
       <c r="E57" s="3">
-        <v>3199.0</v>
-      </c>
-      <c r="G57" s="6" t="s">
-        <v>17</v>
+        <v>1645.0</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>11</v>
@@ -1274,15 +1310,15 @@
         <v>15</v>
       </c>
       <c r="E58" s="3">
-        <v>3699.0</v>
+        <v>2145.0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>12</v>
@@ -1291,15 +1327,15 @@
         <v>15</v>
       </c>
       <c r="E59" s="3">
-        <v>4299.0</v>
+        <v>2645.0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>13</v>
@@ -1308,24 +1344,24 @@
         <v>15</v>
       </c>
       <c r="E60" s="3">
-        <v>4799.0</v>
+        <v>3145.0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E62" s="3">
-        <v>2435.0</v>
+        <v>2489.0</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>10</v>
@@ -1333,128 +1369,1061 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E63" s="3">
-        <v>2935.0</v>
+        <v>3389.0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E64" s="3">
-        <v>3435.0</v>
+        <v>4049.0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E65" s="3">
-        <v>3935.0</v>
+        <v>4949.0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E67" s="3">
-        <v>2689.0</v>
-      </c>
-      <c r="G67" s="4" t="s">
-        <v>10</v>
+        <v>2449.0</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E68" s="3">
-        <v>3589.0</v>
+        <v>2949.0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E69" s="3">
-        <v>4249.0</v>
+        <v>3599.0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E70" s="3">
+        <v>4099.0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E72" s="3">
+        <v>1949.0</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E73" s="3">
+        <v>2449.0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E74" s="3">
+        <v>3099.0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E75" s="3">
+        <v>3599.0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B77" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E70" s="3">
+      <c r="C77" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E77" s="3">
+        <v>2689.0</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E78" s="3">
+        <v>3589.0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E79" s="3">
+        <v>4249.0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E80" s="3">
         <v>5149.0</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E82" s="3">
+        <v>2160.0</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E83" s="3">
+        <v>2660.0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E84" s="3">
+        <v>3160.0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E85" s="3">
+        <v>3660.0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E87" s="3">
+        <v>2199.0</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E88" s="3">
+        <v>2699.0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E89" s="3">
+        <v>3199.0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E90" s="3">
+        <v>3699.0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E92" s="3">
+        <v>2249.0</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E93" s="3">
+        <v>2749.0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E94" s="3">
+        <v>3399.0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E95" s="3">
+        <v>3899.0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E97" s="3">
+        <v>1799.0</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E98" s="3">
+        <v>2299.0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E99" s="3">
+        <v>2799.0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E100" s="3">
+        <v>3299.0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E102" s="3">
+        <v>1799.0</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E103" s="3">
+        <v>2299.0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E104" s="3">
+        <v>2799.0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E105" s="3">
+        <v>3299.0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E107" s="3">
+        <v>2179.0</v>
+      </c>
+      <c r="G107" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E108" s="3">
+        <v>2679.0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E109" s="3">
+        <v>3329.0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E110" s="3">
+        <v>3729.0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E112" s="3">
+        <v>2379.0</v>
+      </c>
+      <c r="G112" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E113" s="3">
+        <v>2879.0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E114" s="3">
+        <v>3529.0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E115" s="3">
+        <v>3929.0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E117" s="3">
+        <v>2635.0</v>
+      </c>
+      <c r="G117" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E118" s="3">
+        <v>3135.0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E119" s="3">
+        <v>3635.0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E120" s="3">
+        <v>4135.0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E122" s="3">
+        <v>3199.0</v>
+      </c>
+      <c r="G122" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E123" s="3">
+        <v>3699.0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E124" s="3">
+        <v>4299.0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E125" s="3">
+        <v>4799.0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E127" s="3">
+        <v>2435.0</v>
+      </c>
+      <c r="G127" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E128" s="3">
+        <v>2935.0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E129" s="3">
+        <v>3435.0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E130" s="3">
+        <v>3935.0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E132" s="3">
+        <v>2689.0</v>
+      </c>
+      <c r="G132" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E133" s="3">
+        <v>3589.0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E134" s="3">
+        <v>4249.0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E135" s="3">
+        <v>5149.0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="27">
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="G7:G10"/>
+    <mergeCell ref="G12:G15"/>
+    <mergeCell ref="G17:G20"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="G27:G30"/>
+    <mergeCell ref="G32:G35"/>
     <mergeCell ref="G37:G40"/>
     <mergeCell ref="G42:G45"/>
     <mergeCell ref="G47:G50"/>
@@ -1462,13 +2431,19 @@
     <mergeCell ref="G57:G60"/>
     <mergeCell ref="G62:G65"/>
     <mergeCell ref="G67:G70"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="G7:G10"/>
-    <mergeCell ref="G12:G15"/>
-    <mergeCell ref="G17:G20"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="G27:G30"/>
-    <mergeCell ref="G32:G35"/>
+    <mergeCell ref="G107:G110"/>
+    <mergeCell ref="G112:G115"/>
+    <mergeCell ref="G117:G120"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="G127:G130"/>
+    <mergeCell ref="G132:G135"/>
+    <mergeCell ref="G72:G75"/>
+    <mergeCell ref="G77:G80"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="G87:G90"/>
+    <mergeCell ref="G92:G95"/>
+    <mergeCell ref="G97:G100"/>
+    <mergeCell ref="G102:G105"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>